<commit_message>
ajouter des fonctions avancées+API+Ameliorer les interfaces
</commit_message>
<xml_diff>
--- a/PIDEV-integrationjava/utilisateurs.xlsx
+++ b/PIDEV-integrationjava/utilisateurs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -156,6 +156,30 @@
   </si>
   <si>
     <t>2025-04-24</t>
+  </si>
+  <si>
+    <t>rabi3</t>
+  </si>
+  <si>
+    <t>rab3oun</t>
+  </si>
+  <si>
+    <t>rabi3@gmail.com</t>
+  </si>
+  <si>
+    <t>2025-04-26</t>
+  </si>
+  <si>
+    <t>abufasaaa</t>
+  </si>
+  <si>
+    <t>balboul</t>
+  </si>
+  <si>
+    <t>balboul@gmail.com</t>
+  </si>
+  <si>
+    <t>2025-04-27</t>
   </si>
 </sst>
 </file>
@@ -163,7 +187,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -171,16 +195,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="58"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="58"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -188,267 +228,329 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="3.26953125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="3.3046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="23.5390625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.7265625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="27.984375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="52.3828125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="16.8515625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="18.84765625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s" s="1">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s" s="1">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s" s="1">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s" s="1">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n" s="0">
+      <c r="A2" t="n" s="2">
         <v>1.0</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n" s="0">
+      <c r="A3" t="n" s="2">
         <v>3.0</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s" s="2">
         <v>11</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F3" t="s" s="0">
+      <c r="F3" t="s" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n" s="0">
+      <c r="A4" t="n" s="2">
         <v>5.0</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="D4" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="E4" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="F4" t="s" s="0">
+      <c r="F4" t="s" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n" s="0">
+      <c r="A5" t="n" s="2">
         <v>9.0</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="E5" t="s" s="0">
+      <c r="E5" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="F5" t="s" s="0">
+      <c r="F5" t="s" s="2">
         <v>22</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n" s="0">
+      <c r="A6" t="n" s="2">
         <v>10.0</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E6" t="s" s="0">
+      <c r="E6" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="F6" t="s" s="0">
+      <c r="F6" t="s" s="2">
         <v>22</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n" s="0">
+      <c r="A7" t="n" s="2">
         <v>20.0</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="E7" t="s" s="0">
+      <c r="E7" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="F7" t="s" s="0">
+      <c r="F7" t="s" s="2">
         <v>31</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n" s="0">
+      <c r="A8" t="n" s="2">
         <v>21.0</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="C8" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="D8" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="E8" t="s" s="0">
+      <c r="E8" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="F8" t="s" s="0">
+      <c r="F8" t="s" s="2">
         <v>35</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n" s="0">
+      <c r="A9" t="n" s="2">
         <v>23.0</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="C9" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="D9" t="s" s="0">
+      <c r="D9" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="E9" t="s" s="0">
+      <c r="E9" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="F9" t="s" s="0">
+      <c r="F9" t="s" s="2">
         <v>35</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n" s="0">
+      <c r="A10" t="n" s="2">
         <v>24.0</v>
       </c>
-      <c r="B10" t="s" s="0">
+      <c r="B10" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="C10" t="s" s="0">
+      <c r="C10" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="D10" t="s" s="0">
+      <c r="D10" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="E10" t="s" s="0">
+      <c r="E10" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="F10" t="s" s="0">
+      <c r="F10" t="s" s="2">
         <v>35</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n" s="0">
+      <c r="A11" t="n" s="2">
         <v>25.0</v>
       </c>
-      <c r="B11" t="s" s="0">
+      <c r="B11" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="C11" t="s" s="0">
+      <c r="C11" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="D11" t="s" s="0">
+      <c r="D11" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="E11" t="s" s="0">
+      <c r="E11" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="F11" t="s" s="0">
+      <c r="F11" t="s" s="2">
         <v>35</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n" s="0">
+      <c r="A12" t="n" s="2">
         <v>29.0</v>
       </c>
-      <c r="B12" t="s" s="0">
+      <c r="B12" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="C12" t="s" s="0">
+      <c r="C12" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="D12" t="s" s="0">
+      <c r="D12" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="E12" t="s" s="0">
+      <c r="E12" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="F12" t="s" s="0">
+      <c r="F12" t="s" s="2">
         <v>47</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="B13" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="C13" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="D13" t="s" s="2">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s" s="2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="D14" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s" s="2">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s" s="2">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>